<commit_message>
Five slot design improvements
</commit_message>
<xml_diff>
--- a/V1.0/Bill Of Materials CartToolFiveSlot - Routed.csv.xlsx
+++ b/V1.0/Bill Of Materials CartToolFiveSlot - Routed.csv.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="116">
   <si>
     <t xml:space="preserve">﻿Category</t>
   </si>
@@ -91,45 +91,63 @@
     <t xml:space="preserve">Resistors</t>
   </si>
   <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R1,R2,R3,R5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PR02000202000JR500</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.sg/ProductDetail/Vishay-BC-Components/PR02000202000JR500?qs=LCMWAU1DZcxqc7IWkiXYPw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generic resistor symbol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RES40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R4,R54</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G6L-1P-DC5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.sg/ProductDetail/Omron-Electronics/G6L-1P-DC5?qs=sQVrL4YZhsQ8oRG2i%2FXEVA%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RELAY TELECOM SPST 1A 5VDC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">G6L1PDC5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">48</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R6,R7,R8,R9,R10,R11,R12,R13,R14,R15,R16,R17,R18,R19,R20,R21,R22,R23,R24,R25,R26,R27,R28,R29,R30,R31,R32,R33,R34,R35,R36,R37,R38,R39,R40,R41,R42,R43,R44,R45,R46,R47,R48,R49,R50,R51,R52,R53</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CR0805-JW-103ELF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.sg/ProductDetail/Bourns/CR0805-JW-103ELF?qs=3T0Ne7aOLxCPz7FUKqmeVw%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SMD 0805 thick film resistor 10k +/-5% 0.125W +/-200ppm/C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RESC2012X60N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Integrated Circuits</t>
+  </si>
+  <si>
     <t xml:space="preserve">5</t>
   </si>
   <si>
-    <t xml:space="preserve">R1,R2,R3,R4,R5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PR02000202000JR500</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mouser.sg/ProductDetail/Vishay-BC-Components/PR02000202000JR500?qs=LCMWAU1DZcxqc7IWkiXYPw%3D%3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generic resistor symbol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RES40</t>
-  </si>
-  <si>
-    <t xml:space="preserve">48</t>
-  </si>
-  <si>
-    <t xml:space="preserve">R6,R7,R8,R9,R10,R11,R12,R13,R14,R15,R16,R17,R18,R19,R20,R21,R22,R23,R24,R25,R26,R27,R28,R29,R30,R31,R32,R33,R34,R35,R36,R37,R38,R39,R40,R41,R42,R43,R44,R45,R46,R47,R48,R49,R50,R51,R52,R53</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CR0805-JW-103ELF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.mouser.sg/ProductDetail/Bourns/CR0805-JW-103ELF?qs=3T0Ne7aOLxCPz7FUKqmeVw%3D%3D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SMD 0805 thick film resistor 10k +/-5% 0.125W +/-200ppm/C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RESC2012X60N</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Integrated Circuits</t>
-  </si>
-  <si>
     <t xml:space="preserve">U1,U8,U11,U15,U18</t>
   </si>
   <si>
@@ -145,9 +163,6 @@
     <t xml:space="preserve">SOIC127P1030X265-20N-CAP</t>
   </si>
   <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
     <t xml:space="preserve">U2,U3,U4,U5</t>
   </si>
   <si>
@@ -208,6 +223,36 @@
     <t xml:space="preserve">TL59AF160Q</t>
   </si>
   <si>
+    <t xml:space="preserve">U21</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ULN2803CDWR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.sg/ProductDetail/Texas-Instruments/ULN2803CDWR?qs=vvQtp7zwQdMA2JP56CSJyQ%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bipolar (BJT) Transistor Array 8 NPN Darlington 50V 500mA Surface Mount 20-SOIC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOIC127P1030X265-20N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SN74LS138DR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS138DR?qs=SL3LIuy2dWwYDw%252Bne7f7PA%3D%3D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-Line to 8-Line Decoders/Demultiplexers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOIC127P600X175-16N-CAP</t>
+  </si>
+  <si>
     <t xml:space="preserve">U492</t>
   </si>
   <si>
@@ -247,7 +292,7 @@
     <t xml:space="preserve">Diodes</t>
   </si>
   <si>
-    <t xml:space="preserve">D1,D2,D3,D4,D5</t>
+    <t xml:space="preserve">D1,D2,D3,D5</t>
   </si>
   <si>
     <t xml:space="preserve">C503C-RCN-CYCZaAA1</t>
@@ -313,7 +358,7 @@
     <t xml:space="preserve">CONN-SIL2</t>
   </si>
   <si>
-    <t xml:space="preserve">20</t>
+    <t xml:space="preserve">21</t>
   </si>
   <si>
     <t xml:space="preserve">One 100nF (0.1uF) capacitor for SMT ICs marked with extra SDC near pin 1</t>
@@ -611,7 +656,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="13.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.29"/>
@@ -732,22 +777,22 @@
         <v>22</v>
       </c>
       <c r="B5" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" s="0" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="D5" s="0" t="s">
         <v>30</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="F5" s="0" t="s">
         <v>32</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="G5" s="0" t="s">
         <v>33</v>
-      </c>
-      <c r="G5" s="0" t="s">
-        <v>34</v>
       </c>
       <c r="H5" s="0" t="s">
         <v>15</v>
@@ -755,25 +800,25 @@
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="0" t="s">
         <v>35</v>
       </c>
-      <c r="B6" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="0" t="s">
+      <c r="D6" s="0" t="s">
         <v>36</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="0" t="s">
         <v>38</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="G6" s="0" t="s">
         <v>39</v>
-      </c>
-      <c r="G6" s="0" t="s">
-        <v>40</v>
       </c>
       <c r="H6" s="0" t="s">
         <v>15</v>
@@ -781,7 +826,7 @@
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B7" s="0" t="s">
         <v>41</v>
@@ -807,10 +852,10 @@
     </row>
     <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>47</v>
@@ -833,25 +878,25 @@
     </row>
     <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B9" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="D9" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="F9" s="0" t="s">
         <v>55</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="G9" s="0" t="s">
         <v>56</v>
-      </c>
-      <c r="G9" s="0" t="s">
-        <v>40</v>
       </c>
       <c r="H9" s="0" t="s">
         <v>15</v>
@@ -859,25 +904,25 @@
     </row>
     <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>16</v>
+        <v>57</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F10" s="0" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G10" s="0" t="s">
-        <v>61</v>
+        <v>46</v>
       </c>
       <c r="H10" s="0" t="s">
         <v>15</v>
@@ -885,7 +930,7 @@
     </row>
     <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B11" s="0" t="s">
         <v>16</v>
@@ -911,25 +956,25 @@
     </row>
     <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C12" s="0" t="s">
         <v>67</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="D12" s="0" t="s">
         <v>68</v>
       </c>
-      <c r="C12" s="0" t="s">
+      <c r="E12" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="F12" s="0" t="s">
         <v>70</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="G12" s="0" t="s">
         <v>71</v>
-      </c>
-      <c r="F12" s="0" t="s">
-        <v>72</v>
-      </c>
-      <c r="G12" s="0" t="s">
-        <v>73</v>
       </c>
       <c r="H12" s="0" t="s">
         <v>15</v>
@@ -937,25 +982,25 @@
     </row>
     <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="E13" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C13" s="0" t="s">
+      <c r="F13" s="0" t="s">
         <v>75</v>
       </c>
-      <c r="D13" s="0" t="s">
+      <c r="G13" s="0" t="s">
         <v>76</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F13" s="0" t="s">
-        <v>78</v>
-      </c>
-      <c r="G13" s="0" t="s">
-        <v>79</v>
       </c>
       <c r="H13" s="0" t="s">
         <v>15</v>
@@ -963,25 +1008,25 @@
     </row>
     <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F14" s="0" t="s">
         <v>80</v>
       </c>
-      <c r="B14" s="0" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14" s="0" t="s">
+      <c r="G14" s="0" t="s">
         <v>81</v>
-      </c>
-      <c r="D14" s="0" t="s">
-        <v>82</v>
-      </c>
-      <c r="E14" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="F14" s="0" t="s">
-        <v>84</v>
-      </c>
-      <c r="G14" s="0" t="s">
-        <v>85</v>
       </c>
       <c r="H14" s="0" t="s">
         <v>15</v>
@@ -989,51 +1034,51 @@
     </row>
     <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>16</v>
+        <v>83</v>
       </c>
       <c r="C15" s="0" t="s">
+        <v>84</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>85</v>
+      </c>
+      <c r="E15" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="F15" s="0" t="s">
         <v>87</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="G15" s="0" t="s">
         <v>88</v>
       </c>
-      <c r="F15" s="0" t="s">
-        <v>89</v>
-      </c>
-      <c r="G15" s="0" t="s">
-        <v>90</v>
-      </c>
       <c r="H15" s="0" t="s">
-        <v>91</v>
+        <v>15</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="B16" s="0" t="s">
         <v>23</v>
       </c>
       <c r="C16" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="D16" s="0" t="s">
+        <v>91</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="F16" s="0" t="s">
         <v>93</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="G16" s="0" t="s">
         <v>94</v>
-      </c>
-      <c r="F16" s="0" t="s">
-        <v>95</v>
-      </c>
-      <c r="G16" s="0" t="s">
-        <v>96</v>
       </c>
       <c r="H16" s="0" t="s">
         <v>15</v>
@@ -1041,19 +1086,19 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>8</v>
+        <v>95</v>
       </c>
       <c r="B17" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C17" s="0" t="s">
+        <v>96</v>
+      </c>
+      <c r="D17" s="0" t="s">
         <v>97</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="E17" s="1" t="s">
         <v>98</v>
-      </c>
-      <c r="D17" s="0" t="s">
-        <v>18</v>
-      </c>
-      <c r="E17" s="1" t="s">
-        <v>19</v>
       </c>
       <c r="F17" s="0" t="s">
         <v>99</v>
@@ -1062,6 +1107,84 @@
         <v>100</v>
       </c>
       <c r="H17" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>101</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>102</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>104</v>
+      </c>
+      <c r="G18" s="0" t="s">
+        <v>105</v>
+      </c>
+      <c r="H18" s="0" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>95</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>107</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>108</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="0" t="s">
+        <v>110</v>
+      </c>
+      <c r="G19" s="0" t="s">
+        <v>111</v>
+      </c>
+      <c r="H19" s="0" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>112</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>113</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>18</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" s="0" t="s">
+        <v>114</v>
+      </c>
+      <c r="G20" s="0" t="s">
+        <v>115</v>
+      </c>
+      <c r="H20" s="0" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1070,19 +1193,22 @@
     <hyperlink ref="E2" r:id="rId1" display="https://www.mouser.sg/ProductDetail/Panasonic/EEU-FR1E471YB?qs=n1SRcuzDZT1JwIghP%252BP6vA%3D%3D"/>
     <hyperlink ref="E3" r:id="rId2" display="https://www.mouser.sg/ProductDetail/Samsung-Electro-Mechanics/CL05B104KO5NNNC?qs=hqM3L16%252BxlfT2SKOuAUq6Q%3D%3D"/>
     <hyperlink ref="E4" r:id="rId3" display="https://www.mouser.sg/ProductDetail/Vishay-BC-Components/PR02000202000JR500?qs=LCMWAU1DZcxqc7IWkiXYPw%3D%3D"/>
-    <hyperlink ref="E5" r:id="rId4" display="https://www.mouser.sg/ProductDetail/Bourns/CR0805-JW-103ELF?qs=3T0Ne7aOLxCPz7FUKqmeVw%3D%3D"/>
-    <hyperlink ref="E6" r:id="rId5" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS374DWR?qs=SL3LIuy2dWx46uWPzrGxvw%3D%3D"/>
-    <hyperlink ref="E7" r:id="rId6" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS273NSR?qs=SL3LIuy2dWxsq%2FCTeVMKZg%3D%3D"/>
-    <hyperlink ref="E8" r:id="rId7" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS04DR?qs=SL3LIuy2dWzOhepjTMFpMg%3D%3D"/>
-    <hyperlink ref="E9" r:id="rId8" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS373DWR?qs=4FFjqLL55bR6x3WZek%252BFgQ%3D%3D"/>
-    <hyperlink ref="E10" r:id="rId9" display="https://www.mouser.sg/ProductDetail/E-Switch/TL59F260Q?qs=QtyuwXswaQiASDh1C66FNg%3D%3D"/>
-    <hyperlink ref="E11" r:id="rId10" display="https://www.mouser.sg/ProductDetail/Analog-Devices/ADM709LARZ?qs=BpaRKvA4VqHy5OxrBQwb0w%3D%3D"/>
-    <hyperlink ref="E12" r:id="rId11" display="https://www.mouser.sg/ProductDetail/onsemi-Fairchild/BSS138?qs=HK%252BeIG1iaahCeqBvjB4arg%3D%3D"/>
-    <hyperlink ref="E13" r:id="rId12" display="https://www.mouser.sg/ProductDetail/Cree-LED/C503C-RCN-CYCZaAA1?qs=mwfrHz%252BSIuGPYiPc7W1Mew%3D%3D"/>
-    <hyperlink ref="E14" r:id="rId13" display="https://www.mouser.com/ProductDetail/TE-Connectivity/5530843-4?qs=CWN9I2qbSLsRSJz%252BQBuIeg%3D%3D"/>
-    <hyperlink ref="E15" r:id="rId14" display="https://www.mouser.sg/ProductDetail/3M-Electronic-Solutions-Division/929975-01-20-RK?qs=4V84emjyG36rTUkvYfpt0A%3D%3D"/>
-    <hyperlink ref="E16" r:id="rId15" display="https://www.mouser.sg/ProductDetail/3M-Electronic-Solutions-Division/929850-01-02-10?qs=sGAEpiMZZMs%252BGHln7q6pm6DQXoV0bF8fKj%2FScW6NT6k%3D"/>
-    <hyperlink ref="E17" r:id="rId16" display="https://www.mouser.sg/ProductDetail/Samsung-Electro-Mechanics/CL05B104KO5NNNC?qs=hqM3L16%252BxlfT2SKOuAUq6Q%3D%3D"/>
+    <hyperlink ref="E5" r:id="rId4" display="https://www.mouser.sg/ProductDetail/Omron-Electronics/G6L-1P-DC5?qs=sQVrL4YZhsQ8oRG2i%2FXEVA%3D%3D"/>
+    <hyperlink ref="E6" r:id="rId5" display="https://www.mouser.sg/ProductDetail/Bourns/CR0805-JW-103ELF?qs=3T0Ne7aOLxCPz7FUKqmeVw%3D%3D"/>
+    <hyperlink ref="E7" r:id="rId6" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS374DWR?qs=SL3LIuy2dWx46uWPzrGxvw%3D%3D"/>
+    <hyperlink ref="E8" r:id="rId7" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS273NSR?qs=SL3LIuy2dWxsq%2FCTeVMKZg%3D%3D"/>
+    <hyperlink ref="E9" r:id="rId8" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS04DR?qs=SL3LIuy2dWzOhepjTMFpMg%3D%3D"/>
+    <hyperlink ref="E10" r:id="rId9" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS373DWR?qs=4FFjqLL55bR6x3WZek%252BFgQ%3D%3D"/>
+    <hyperlink ref="E11" r:id="rId10" display="https://www.mouser.sg/ProductDetail/E-Switch/TL59F260Q?qs=QtyuwXswaQiASDh1C66FNg%3D%3D"/>
+    <hyperlink ref="E12" r:id="rId11" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/ULN2803CDWR?qs=vvQtp7zwQdMA2JP56CSJyQ%3D%3D"/>
+    <hyperlink ref="E13" r:id="rId12" display="https://www.mouser.sg/ProductDetail/Texas-Instruments/SN74LS138DR?qs=SL3LIuy2dWwYDw%252Bne7f7PA%3D%3D"/>
+    <hyperlink ref="E14" r:id="rId13" display="https://www.mouser.sg/ProductDetail/Analog-Devices/ADM709LARZ?qs=BpaRKvA4VqHy5OxrBQwb0w%3D%3D"/>
+    <hyperlink ref="E15" r:id="rId14" display="https://www.mouser.sg/ProductDetail/onsemi-Fairchild/BSS138?qs=HK%252BeIG1iaahCeqBvjB4arg%3D%3D"/>
+    <hyperlink ref="E16" r:id="rId15" display="https://www.mouser.sg/ProductDetail/Cree-LED/C503C-RCN-CYCZaAA1?qs=mwfrHz%252BSIuGPYiPc7W1Mew%3D%3D"/>
+    <hyperlink ref="E17" r:id="rId16" display="https://www.mouser.com/ProductDetail/TE-Connectivity/5530843-4?qs=CWN9I2qbSLsRSJz%252BQBuIeg%3D%3D"/>
+    <hyperlink ref="E18" r:id="rId17" display="https://www.mouser.sg/ProductDetail/3M-Electronic-Solutions-Division/929975-01-20-RK?qs=4V84emjyG36rTUkvYfpt0A%3D%3D"/>
+    <hyperlink ref="E19" r:id="rId18" display="https://www.mouser.sg/ProductDetail/3M-Electronic-Solutions-Division/929850-01-02-10?qs=sGAEpiMZZMs%252BGHln7q6pm6DQXoV0bF8fKj%2FScW6NT6k%3D"/>
+    <hyperlink ref="E20" r:id="rId19" display="https://www.mouser.sg/ProductDetail/Samsung-Electro-Mechanics/CL05B104KO5NNNC?qs=hqM3L16%252BxlfT2SKOuAUq6Q%3D%3D"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>